<commit_message>
updated Code of Cosmohub backend till 04062025
</commit_message>
<xml_diff>
--- a/assets/Import client.xlsx
+++ b/assets/Import client.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28129"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28429"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Node_JS_Boot\PSoft work\CosmoHub\Documents\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Node_JS_Boot\PSoft work\CosmoHub\server\assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{678C0384-B0CF-4EDE-B56C-0874791A4480}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AE74EDC1-165D-4459-99DE-26F4D867A113}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{881B1A0A-4608-41B5-92DB-5F7684B139AB}"/>
   </bookViews>
@@ -75,9 +75,6 @@
     <t>Kamothe</t>
   </si>
   <si>
-    <t>Pravin12 Karande</t>
-  </si>
-  <si>
     <t>Pravin13 Karande</t>
   </si>
   <si>
@@ -112,6 +109,9 @@
   </si>
   <si>
     <t>Maharashtra</t>
+  </si>
+  <si>
+    <t>ira pise</t>
   </si>
 </sst>
 </file>
@@ -495,7 +495,7 @@
         <v>14</v>
       </c>
       <c r="F1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G1" t="s">
         <v>4</v>
@@ -504,13 +504,13 @@
         <v>5</v>
       </c>
       <c r="I1" t="s">
+        <v>23</v>
+      </c>
+      <c r="J1" t="s">
         <v>24</v>
       </c>
-      <c r="J1" t="s">
+      <c r="K1" t="s">
         <v>25</v>
-      </c>
-      <c r="K1" t="s">
-        <v>26</v>
       </c>
       <c r="L1" t="s">
         <v>6</v>
@@ -521,13 +521,13 @@
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>16</v>
+        <v>28</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>13</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D2" t="s">
         <v>8</v>
@@ -545,10 +545,10 @@
         <v>0</v>
       </c>
       <c r="I2" t="s">
+        <v>26</v>
+      </c>
+      <c r="J2" t="s">
         <v>27</v>
-      </c>
-      <c r="J2" t="s">
-        <v>28</v>
       </c>
       <c r="K2" t="s">
         <v>15</v>
@@ -562,13 +562,13 @@
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B3" s="1" t="s">
         <v>13</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D3" t="s">
         <v>8</v>
@@ -586,10 +586,10 @@
         <v>0</v>
       </c>
       <c r="I3" t="s">
+        <v>26</v>
+      </c>
+      <c r="J3" t="s">
         <v>27</v>
-      </c>
-      <c r="J3" t="s">
-        <v>28</v>
       </c>
       <c r="K3" t="s">
         <v>15</v>
@@ -603,13 +603,13 @@
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B4" s="1" t="s">
         <v>13</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D4" t="s">
         <v>8</v>
@@ -627,10 +627,10 @@
         <v>0</v>
       </c>
       <c r="I4" t="s">
+        <v>26</v>
+      </c>
+      <c r="J4" t="s">
         <v>27</v>
-      </c>
-      <c r="J4" t="s">
-        <v>28</v>
       </c>
       <c r="K4" t="s">
         <v>15</v>
@@ -644,13 +644,13 @@
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B5" s="1" t="s">
         <v>13</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D5" t="s">
         <v>8</v>
@@ -668,10 +668,10 @@
         <v>0</v>
       </c>
       <c r="I5" t="s">
+        <v>26</v>
+      </c>
+      <c r="J5" t="s">
         <v>27</v>
-      </c>
-      <c r="J5" t="s">
-        <v>28</v>
       </c>
       <c r="K5" t="s">
         <v>15</v>
@@ -685,13 +685,13 @@
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B6" s="1" t="s">
         <v>13</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D6" t="s">
         <v>8</v>
@@ -709,10 +709,10 @@
         <v>0</v>
       </c>
       <c r="I6" t="s">
+        <v>26</v>
+      </c>
+      <c r="J6" t="s">
         <v>27</v>
-      </c>
-      <c r="J6" t="s">
-        <v>28</v>
       </c>
       <c r="K6" t="s">
         <v>15</v>
@@ -726,13 +726,13 @@
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B7" s="1" t="s">
         <v>13</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D7" t="s">
         <v>8</v>
@@ -750,10 +750,10 @@
         <v>0</v>
       </c>
       <c r="I7" t="s">
+        <v>26</v>
+      </c>
+      <c r="J7" t="s">
         <v>27</v>
-      </c>
-      <c r="J7" t="s">
-        <v>28</v>
       </c>
       <c r="K7" t="s">
         <v>15</v>

</xml_diff>